<commit_message>
Fallando la fecha del body
</commit_message>
<xml_diff>
--- a/data/resume.xlsx
+++ b/data/resume.xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="107">
   <si>
     <t>date</t>
   </si>
@@ -285,6 +285,81 @@
   </si>
   <si>
     <t>2025-10-03 17:59:37</t>
+  </si>
+  <si>
+    <t>2025-10-03 18:10:43</t>
+  </si>
+  <si>
+    <t>2025-10-03 18:10:44</t>
+  </si>
+  <si>
+    <t>2025-10-03 18:10:45</t>
+  </si>
+  <si>
+    <t>2025-10-06 12:38:24</t>
+  </si>
+  <si>
+    <t>2025-10-06 12:38:25</t>
+  </si>
+  <si>
+    <t>2025-10-06 12:38:26</t>
+  </si>
+  <si>
+    <t>10/03/2025</t>
+  </si>
+  <si>
+    <t>2025-10-06 20:17:08</t>
+  </si>
+  <si>
+    <t>2025-10-06 20:17:09</t>
+  </si>
+  <si>
+    <t>2025-10-06 20:17:10</t>
+  </si>
+  <si>
+    <t>2025-10-06 20:17:44</t>
+  </si>
+  <si>
+    <t>2025-10-06 20:17:45</t>
+  </si>
+  <si>
+    <t>2025-10-06 20:17:46</t>
+  </si>
+  <si>
+    <t>2025-10-06 20:17:55</t>
+  </si>
+  <si>
+    <t>2025-10-06 20:17:56</t>
+  </si>
+  <si>
+    <t>2025-10-06 20:17:57</t>
+  </si>
+  <si>
+    <t>2025-10-06 20:18:22</t>
+  </si>
+  <si>
+    <t>2025-10-06 20:18:23</t>
+  </si>
+  <si>
+    <t>2025-10-06 20:18:24</t>
+  </si>
+  <si>
+    <t>2025-10-06 20:19:48</t>
+  </si>
+  <si>
+    <t>2025-10-06 20:19:50</t>
+  </si>
+  <si>
+    <t>2025-10-06 20:19:51</t>
+  </si>
+  <si>
+    <t>2025-10-06 20:21:20</t>
+  </si>
+  <si>
+    <t>2025-10-06 20:21:21</t>
+  </si>
+  <si>
+    <t>2025-10-06 20:21:22</t>
   </si>
 </sst>
 </file>
@@ -1091,7 +1166,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D91"/>
+  <dimension ref="A1:D119"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.73046875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col customWidth="1" max="1" min="1" width="24.19921875"/>
@@ -2374,6 +2449,390 @@
         <v>8</v>
       </c>
     </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A92" t="s">
+        <v>82</v>
+      </c>
+      <c r="B92" t="s">
+        <v>65</v>
+      </c>
+      <c r="C92" t="s">
+        <v>17</v>
+      </c>
+      <c r="D92">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A93" t="s">
+        <v>83</v>
+      </c>
+      <c r="B93" t="s">
+        <v>65</v>
+      </c>
+      <c r="C93" t="s">
+        <v>18</v>
+      </c>
+      <c r="D93">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A94" t="s">
+        <v>83</v>
+      </c>
+      <c r="B94" t="s">
+        <v>65</v>
+      </c>
+      <c r="C94" t="s">
+        <v>19</v>
+      </c>
+      <c r="D94">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A95" t="s">
+        <v>83</v>
+      </c>
+      <c r="B95" t="s">
+        <v>65</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A96" t="s">
+        <v>83</v>
+      </c>
+      <c r="B96" t="s">
+        <v>65</v>
+      </c>
+      <c r="C96" t="s">
+        <v>21</v>
+      </c>
+      <c r="D96">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A97" t="s">
+        <v>84</v>
+      </c>
+      <c r="B97" t="s">
+        <v>65</v>
+      </c>
+      <c r="C97" t="s">
+        <v>22</v>
+      </c>
+      <c r="D97">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A98" t="s">
+        <v>85</v>
+      </c>
+      <c r="B98" t="s">
+        <v>88</v>
+      </c>
+      <c r="C98" t="s">
+        <v>20</v>
+      </c>
+      <c r="D98">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A99" t="s">
+        <v>86</v>
+      </c>
+      <c r="B99" t="s">
+        <v>88</v>
+      </c>
+      <c r="C99" t="s">
+        <v>21</v>
+      </c>
+      <c r="D99">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A100" t="s">
+        <v>87</v>
+      </c>
+      <c r="B100" t="s">
+        <v>88</v>
+      </c>
+      <c r="C100" t="s">
+        <v>22</v>
+      </c>
+      <c r="D100">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A101" t="s">
+        <v>89</v>
+      </c>
+      <c r="B101" t="s">
+        <v>88</v>
+      </c>
+      <c r="C101" t="s">
+        <v>20</v>
+      </c>
+      <c r="D101">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A102" t="s">
+        <v>90</v>
+      </c>
+      <c r="B102" t="s">
+        <v>88</v>
+      </c>
+      <c r="C102" t="s">
+        <v>21</v>
+      </c>
+      <c r="D102">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A103" t="s">
+        <v>91</v>
+      </c>
+      <c r="B103" t="s">
+        <v>88</v>
+      </c>
+      <c r="C103" t="s">
+        <v>22</v>
+      </c>
+      <c r="D103">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A104" t="s">
+        <v>92</v>
+      </c>
+      <c r="B104" t="s">
+        <v>88</v>
+      </c>
+      <c r="C104" t="s">
+        <v>20</v>
+      </c>
+      <c r="D104">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A105" t="s">
+        <v>93</v>
+      </c>
+      <c r="B105" t="s">
+        <v>88</v>
+      </c>
+      <c r="C105" t="s">
+        <v>21</v>
+      </c>
+      <c r="D105">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A106" t="s">
+        <v>94</v>
+      </c>
+      <c r="B106" t="s">
+        <v>88</v>
+      </c>
+      <c r="C106" t="s">
+        <v>22</v>
+      </c>
+      <c r="D106">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A107" t="s">
+        <v>95</v>
+      </c>
+      <c r="B107" t="s">
+        <v>88</v>
+      </c>
+      <c r="C107" t="s">
+        <v>20</v>
+      </c>
+      <c r="D107">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A108" t="s">
+        <v>96</v>
+      </c>
+      <c r="B108" t="s">
+        <v>88</v>
+      </c>
+      <c r="C108" t="s">
+        <v>21</v>
+      </c>
+      <c r="D108">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A109" t="s">
+        <v>97</v>
+      </c>
+      <c r="B109" t="s">
+        <v>88</v>
+      </c>
+      <c r="C109" t="s">
+        <v>22</v>
+      </c>
+      <c r="D109">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A110" t="s">
+        <v>98</v>
+      </c>
+      <c r="B110" t="s">
+        <v>88</v>
+      </c>
+      <c r="C110" t="s">
+        <v>20</v>
+      </c>
+      <c r="D110">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A111" t="s">
+        <v>99</v>
+      </c>
+      <c r="B111" t="s">
+        <v>88</v>
+      </c>
+      <c r="C111" t="s">
+        <v>21</v>
+      </c>
+      <c r="D111">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A112" t="s">
+        <v>100</v>
+      </c>
+      <c r="B112" t="s">
+        <v>88</v>
+      </c>
+      <c r="C112" t="s">
+        <v>22</v>
+      </c>
+      <c r="D112">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A113" t="s">
+        <v>101</v>
+      </c>
+      <c r="B113" t="s">
+        <v>88</v>
+      </c>
+      <c r="C113" t="s">
+        <v>20</v>
+      </c>
+      <c r="D113">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A114" t="s">
+        <v>102</v>
+      </c>
+      <c r="B114" t="s">
+        <v>88</v>
+      </c>
+      <c r="C114" t="s">
+        <v>21</v>
+      </c>
+      <c r="D114">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A115" t="s">
+        <v>103</v>
+      </c>
+      <c r="B115" t="s">
+        <v>88</v>
+      </c>
+      <c r="C115" t="s">
+        <v>22</v>
+      </c>
+      <c r="D115">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A116" t="s">
+        <v>104</v>
+      </c>
+      <c r="B116" t="s">
+        <v>88</v>
+      </c>
+      <c r="C116" t="s">
+        <v>20</v>
+      </c>
+      <c r="D116">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A117" t="s">
+        <v>105</v>
+      </c>
+      <c r="B117" t="s">
+        <v>88</v>
+      </c>
+      <c r="C117" t="s">
+        <v>21</v>
+      </c>
+      <c r="D117">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A118" t="s">
+        <v>106</v>
+      </c>
+      <c r="B118" t="s">
+        <v>88</v>
+      </c>
+      <c r="C118" t="s">
+        <v>22</v>
+      </c>
+      <c r="D118">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A119"/>
+      <c r="B119"/>
+      <c r="C119"/>
+      <c r="D119"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>

<commit_message>
Poner hora bien en contenedor
</commit_message>
<xml_diff>
--- a/data/resume.xlsx
+++ b/data/resume.xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="104">
   <si>
     <t>date</t>
   </si>
@@ -348,6 +348,9 @@
   </si>
   <si>
     <t>2025-10-08 22:31:42</t>
+  </si>
+  <si>
+    <t>2025-10-08 22:32:41</t>
   </si>
 </sst>
 </file>
@@ -1155,7 +1158,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D92"/>
+  <dimension ref="A1:D93"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.73046875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col customWidth="1" max="1" min="1" width="24.19921875"/>
@@ -2452,6 +2455,20 @@
         <v>15</v>
       </c>
     </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A93" t="s">
+        <v>103</v>
+      </c>
+      <c r="B93" s="1">
+        <v>45933</v>
+      </c>
+      <c r="C93" t="s">
+        <v>21</v>
+      </c>
+      <c r="D93">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>